<commit_message>
Fix Telugu replies and fill demo data for every teacher and for 7 Oct
- Agents get the language name (Telugu, Hindi) instead of the code
- Timetable, syllabus, curriculum and tasks for all teachers; 7 Oct attendance and diary
- Tests clear the log sheets in their workbook copy
</commit_message>
<xml_diff>
--- a/data/school_data.xlsx
+++ b/data/school_data.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -1634,6 +1634,126 @@
         <v>1</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>att-s-nur-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>s-nur-1</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>att-s-ukg-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>s-ukg-1</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>att-s-1-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>s-1-1</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D58" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>att-s-3-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>s-3-1</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D59" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>att-s-5-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>s-5-1</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>att-s-7-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>s-7-1</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D61" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1645,7 +1765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -1833,6 +1953,148 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>Science: write notes on Nutrition in Plants. Maths: practice set 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>diary-s-nur-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>s-nur-1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Napped 40 min, finished lunch, enjoyed sorting blocks by colour.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Colours and shapes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>diary-s-ukg-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>s-ukg-1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Ate all of lunch, joined in the rhyme session, practised writing letter 'C'.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Colours and shapes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>diary-s-1-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>s-1-1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>English: read 'Three Little Pigs' with a parent. Maths: do 5 addition sums in the notebook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>diary-s-3-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>s-3-1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Maths: Give and Take - solve the first 5 sums in the notebook. English: learn the new words from 'Bird Talk'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>diary-s-5-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>s-5-1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Maths: 'How Many Squares?' worksheet - find the area of 3 shapes. English: read 'Teamwork' aloud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>diary-s-7-1-2026-10-07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>s-7-1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Science: draw and label the human digestive system. Maths: Data Handling practice set.</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -3335,6 +3597,1371 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>syl-1-english-01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>A Happy Child</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>syl-1-english-02</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Three Little Pigs</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>syl-1-english-03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>After a Bath</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>syl-1-english-04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>The Bubble, the Straw and the Shoe</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>syl-1-english-05</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>One Little Kitten</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>syl-1-mathematics-01</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Shapes and Space</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>syl-1-mathematics-02</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Numbers from One to Nine</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>syl-1-mathematics-03</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Addition</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>syl-1-mathematics-04</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Subtraction</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>syl-1-mathematics-05</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Numbers from Ten to Twenty</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>syl-3-english-01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Good Morning</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>syl-3-english-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>The Magic Garden</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>syl-3-english-03</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Bird Talk</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>syl-3-english-04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Nina and the Baby Sparrows</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>syl-3-english-05</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Little by Little</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>syl-5-english-01</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Ice-cream Man</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>syl-5-english-02</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Wonderful Waste!</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>syl-5-english-03</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Teamwork</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>syl-5-english-04</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Flying Together</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>syl-5-english-05</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>My Shadow</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>syl-3-evs-01</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Poonam's Day Out</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>syl-3-evs-02</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>The Plant Fairy</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>syl-3-evs-03</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Water O' Water!</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>syl-3-evs-04</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Our First School</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>syl-3-evs-05</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Chhotu's House</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>syl-5-evs-01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Super Senses</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>syl-5-evs-02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>A Snake Charmer's Story</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>syl-5-evs-03</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>From Tasting to Digesting</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>syl-5-evs-04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Mangoes Round the Year</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>syl-5-evs-05</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Seeds and Seeds</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>syl-7-mathematics-01</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Integers</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>syl-7-mathematics-02</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Fractions and Decimals</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>syl-7-mathematics-03</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Data Handling</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>syl-7-mathematics-04</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Simple Equations</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>syl-7-mathematics-05</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Lines and Angles</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3346,7 +4973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3952,6 +5579,1231 @@
       <c r="G17" t="inlineStr">
         <is>
           <t>Acids and bases around us, natural indicators such as litmus and turmeric, and neutralisation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>cur-1-english-01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>A Happy Child</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>A poem about a child who feels happy in the world around them; rhyming words and reading aloud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>cur-1-english-02</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Three Little Pigs</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>The story of three pigs who build houses of straw, sticks and bricks; sequencing and retelling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>cur-1-english-03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>After a Bath</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>A poem about drying off after a bath; action words and body parts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>cur-1-english-04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>The Bubble, the Straw and the Shoe</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>A story about three friends crossing a stream; new words and simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>cur-1-english-05</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>One Little Kitten</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>A counting poem with animals; number words one to ten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>cur-1-mathematics-01</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Shapes and Space</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Inside and outside, near and far, top and bottom, and sorting objects by shape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>cur-1-mathematics-02</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Numbers from One to Nine</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Counting, reading and writing numbers 1 to 9 with objects and pictures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cur-1-mathematics-03</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Addition</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Putting groups together and adding numbers up to 9 using objects and pictures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>cur-1-mathematics-04</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Subtraction</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Taking away from a group and simple subtraction stories up to 9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>cur-1-mathematics-05</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Numbers from Ten to Twenty</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Counting, reading and writing numbers 10 to 20, and tens and ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>cur-3-english-01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Good Morning</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>A poem about the morning and nature; rhyming words and recitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>cur-3-english-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>The Magic Garden</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>A story about flowers that bloom when children care for them; reading and new words.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>cur-3-english-03</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Bird Talk</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>A poem in which birds talk about people; describing words and speaking practice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>cur-3-english-04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Nina and the Baby Sparrows</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>A story about a girl who helps a family of sparrows; reading comprehension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>cur-3-english-05</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Little by Little</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>A poem about how an acorn grows into an oak tree; growth and sequencing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>cur-5-english-01</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Ice-cream Man</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>A poem about the ice-cream seller on a summer day; rhyme and imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>cur-5-english-02</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Wonderful Waste!</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>A story about a cook who makes a new dish (avial) from leftover vegetables; not wasting food.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>cur-5-english-03</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Teamwork</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>A poem about working together; values and recitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>cur-5-english-04</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Flying Together</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>A story about wild geese who learn to listen to the wise old goose; teamwork and good advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>cur-5-english-05</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>My Shadow</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>A poem about a child's shadow that changes size; describing and comparing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>cur-3-evs-01</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Poonam's Day Out</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Animals around us - where they live, what they eat and how they move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>cur-3-evs-02</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>The Plant Fairy</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Plants around us - leaves, flowers, bark and how plants differ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>cur-3-evs-03</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Water O' Water!</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Uses of water, where it comes from, and saving water.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>cur-3-evs-04</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Our First School</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>The family as our first school, family members and what we learn from them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>cur-3-evs-05</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Chhotu's House</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Different kinds of houses and the materials used to build them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>cur-5-evs-01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Super Senses</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>How animals use their senses of sight, smell and hearing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>cur-5-evs-02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>A Snake Charmer's Story</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Snake charmers, their life and how they care for snakes; respecting animals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>cur-5-evs-03</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>From Tasting to Digesting</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Taste, the tongue and how food is digested in the body.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>cur-5-evs-04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>4</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Mangoes Round the Year</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Preserving food - pickles, papad and mango papad - and why food spoils.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>cur-5-evs-05</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>5</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Seeds and Seeds</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>How seeds germinate and how they spread from one place to another.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>cur-7-mathematics-01</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Integers</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Adding, subtracting, multiplying and dividing integers, and their properties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>cur-7-mathematics-02</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Fractions and Decimals</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Multiplying and dividing fractions and decimals in everyday problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>cur-7-mathematics-03</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Data Handling</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Collecting and organising data, mean, median and mode, and bar graphs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>cur-7-mathematics-04</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Simple Equations</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Setting up and solving simple linear equations from word problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>cur-7-mathematics-05</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>CBSE</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>5</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Lines and Angles</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Pairs of angles, parallel lines and transversals.</t>
         </is>
       </c>
     </row>
@@ -4220,7 +7072,6 @@
           <t>holiday</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>School closed.</t>
@@ -4258,7 +7109,6 @@
           <t>ptm</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>PTM for all classes, 9:00 am to 12:00 pm. FA2 report cards will be shared.</t>
@@ -4296,7 +7146,6 @@
           <t>holiday</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>School closed. Classes resume on 22 Oct.</t>
@@ -4334,7 +7183,6 @@
           <t>holiday</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>School closed. Classes resume on 11 Nov.</t>
@@ -4372,7 +7220,6 @@
           <t>event</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Celebrations and cultural programme. Students may come in colour dress.</t>
@@ -4452,7 +7299,6 @@
           <t>event</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Annual Day function at 5:00 pm in the school auditorium. Parents are invited.</t>
@@ -4490,7 +7336,6 @@
           <t>holiday</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>School closed. Classes resume on 4 Jan.</t>
@@ -5631,7 +8476,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>class_teacher</t>
@@ -5723,7 +8567,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>class_teacher</t>
@@ -5783,7 +8626,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>class_teacher</t>
@@ -5811,7 +8653,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>class_teacher</t>
@@ -5839,7 +8680,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>class_teacher</t>
@@ -5931,7 +8771,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>class_teacher</t>
@@ -6109,7 +8948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -6695,6 +9534,1545 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tt-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>t-3</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Nursery</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Circle time</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>R-N1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>tt-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>t-3</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Nursery</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Story and rhymes</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>R-N1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tt-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>t-3</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Nursery</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Play and activity</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>R-N1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tt-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>t-4</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>UKG</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Circle time</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>R-U1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>tt-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>t-4</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>UKG</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Letters and phonics</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>R-U1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tt-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>t-4</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>UKG</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Art and craft</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>R-U1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>tt-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>t-5</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>R-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tt-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>t-5</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>R-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>tt-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>t-5</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>R-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>tt-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>t-5</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>R-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>tt-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>t-5</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>R-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>tt-21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>t-5</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>R-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>tt-22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>t-6</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>R-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>tt-23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>t-6</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>R-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>tt-24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>t-6</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>R-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>tt-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>t-6</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>R-502</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>tt-26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>t-6</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>R-502</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>tt-27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>t-6</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>R-502</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>tt-28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>t-7</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>R-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>tt-29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>t-7</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>R-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>tt-30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>t-7</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>R-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>tt-31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>t-7</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>R-502</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>tt-32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>t-7</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>R-502</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>tt-33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>t-7</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>R-502</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>tt-34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>t-8</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>R-701</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>tt-35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>t-8</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>R-701</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>tt-36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>t-8</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>R-701</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6706,7 +11084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -6909,6 +11287,402 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>task-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>t-3</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Update care logs for Nursery-A</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>task-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>t-3</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Set up the 'Colours and shapes' activity corner</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>task-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>t-4</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Share letter 'C' practice sheet with UKG-A parents</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>task-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>t-4</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Plan the Children's Day performance (UKG-A)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>task-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>t-5</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Check Grade 1-A addition homework</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>task-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>t-5</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Record CCE reading remarks for Grade 1-A</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>task-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>t-6</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Upload FA2 marks for Grade 5-B English</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>task-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>t-6</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Prepare parent-teacher meeting notes (Grade 5-B)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>task-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>t-6</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Correct Grade 3-A reading comprehension sheets</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>task-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>t-7</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Upload FA2 marks for Grade 3 EVS</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>task-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>t-7</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Plan the 'Seeds and Seeds' germination activity for Grade 5-B</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>EVS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>task-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>t-8</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Set an Integers practice worksheet for Grade 7-A</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>task-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>t-8</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Upload FA2 marks for Grade 7 Mathematics</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: save latest school data updates
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/school_data.xlsx
+++ b/data/school_data.xlsx
@@ -6818,7 +6818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -6855,6 +6855,33 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>conversations-bb8ef9d599</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>demo-school</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>g-nur-1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:22:53</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6866,7 +6893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -6906,6 +6933,65 @@
       <c r="F1" s="2" t="inlineStr">
         <is>
           <t>created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>messages-6aa4559c5c</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>conversations-bb8ef9d599</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Was my child present on 6 October?</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:22:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>messages-869efb0060</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>conversations-bb8ef9d599</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>assistant</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>మీ కుమారుడు 6 అక్టోబర్ 2023న హాజరుకాలేదు. ప్రస్తుతం ఈ తేదీకి సంబంధించి రికార్డు లేదు. దయచేసి మరింత సమాచారం కోసం పాఠశాలను సంప్రదించండి.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>daily_update</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:22:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(voice): reply in English or Hindi per turn
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/school_data.xlsx
+++ b/data/school_data.xlsx
@@ -7916,7 +7916,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>te</t>
+          <t>en</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>te</t>
+          <t>en</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>

<commit_message>
Tag saved chat turns with the child and intent so they can be exported for evaluation.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/school_data.xlsx
+++ b/data/school_data.xlsx
@@ -6866,7 +6866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -6906,6 +6906,21 @@
       <c r="F1" s="2" t="inlineStr">
         <is>
           <t>created_at</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>student_id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>intent_source</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>intent_confidence</t>
         </is>
       </c>
     </row>

</xml_diff>